<commit_message>
data(eur): daily refresh 2026-10-07T15:48Z
</commit_message>
<xml_diff>
--- a/logs/eur/raw/de_einzelaufstellung.xlsx
+++ b/logs/eur/raw/de_einzelaufstellung.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="631" xml:space="preserve">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="633" xml:space="preserve">
   <si>
     <r>
       <rPr>
@@ -88,7 +88,7 @@
     <t>2026-06-30</t>
   </si>
   <si>
-    <t>2026-08-31</t>
+    <t>2026-09-30</t>
   </si>
   <si>
     <t>30-year inflation-linked Federal bonds</t>
@@ -1271,6 +1271,12 @@
   </si>
   <si>
     <t>2027-08-18</t>
+  </si>
+  <si>
+    <t>DE000BU0E451</t>
+  </si>
+  <si>
+    <t>2027-09-15</t>
   </si>
   <si>
     <t>Promissory notes</t>
@@ -2710,7 +2716,7 @@
 
 <file path=xl/worksheets/Sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I322"/>
+  <dimension ref="A1:I323"/>
   <sheetFormatPr defaultRowHeight="12.750000" customHeight="true"/>
   <cols>
     <col min="1" max="1" width="125.108739" bestFit="1" customWidth="1"/>
@@ -2726,7 +2732,7 @@
   <sheetData>
     <row r="1" spans="4:4">
       <c r="D1" s="1">
-        <v>46268.36853009</v>
+        <v>46301.33487268</v>
       </c>
     </row>
     <row r="3" spans="7:7">
@@ -3050,7 +3056,7 @@
         <v>4000000000</v>
       </c>
       <c r="I23" s="59">
-        <v>4750000000</v>
+        <v>5500000000</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -3073,7 +3079,7 @@
         <v>4000000000</v>
       </c>
       <c r="I24" s="74">
-        <v>4750000000</v>
+        <v>5500000000</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -3156,7 +3162,7 @@
         <v>13500000000</v>
       </c>
       <c r="I27" s="59">
-        <v>13500000000</v>
+        <v>14250000000</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -3208,7 +3214,7 @@
         <v>43000000000</v>
       </c>
       <c r="I29" s="74">
-        <v>43500000000</v>
+        <v>44250000000</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -3798,7 +3804,7 @@
         <v>28500000000</v>
       </c>
       <c r="I51" s="59">
-        <v>33500000000</v>
+        <v>36000000000</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -3825,7 +3831,7 @@
         <v>486000000000</v>
       </c>
       <c r="I52" s="74">
-        <v>495500000000</v>
+        <v>498000000000</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -3850,7 +3856,7 @@
         <v>10500000000</v>
       </c>
       <c r="I53" s="59">
-        <v>11500000000</v>
+        <v>13500000000</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -3873,7 +3879,7 @@
         <v>10500000000</v>
       </c>
       <c r="I54" s="74">
-        <v>11500000000</v>
+        <v>13500000000</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -4628,7 +4634,7 @@
       <c r="G83" s="52"/>
       <c r="H83" s="52"/>
       <c r="I83" s="59">
-        <v>18000000000</v>
+        <v>23500000000</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -4655,7 +4661,7 @@
         <v>641750000000</v>
       </c>
       <c r="I84" s="74">
-        <v>627250000000</v>
+        <v>632750000000</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -5167,7 +5173,7 @@
       <c r="G104" s="52"/>
       <c r="H104" s="52"/>
       <c r="I104" s="59">
-        <v>12000000000</v>
+        <v>22500000000</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -5194,7 +5200,7 @@
         <v>278500000000</v>
       </c>
       <c r="I105" s="74">
-        <v>290500000000</v>
+        <v>301000000000</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -5352,9 +5358,7 @@
       <c r="H112" s="57">
         <v>19000000000</v>
       </c>
-      <c r="I112" s="59">
-        <v>19000000000</v>
-      </c>
+      <c r="I112" s="58"/>
     </row>
     <row r="113" spans="1:9">
       <c r="A113" s="76"/>
@@ -5547,7 +5551,7 @@
       <c r="G120" s="52"/>
       <c r="H120" s="52"/>
       <c r="I120" s="59">
-        <v>17000000000</v>
+        <v>22000000000</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -5574,7 +5578,7 @@
         <v>158500000000</v>
       </c>
       <c r="I121" s="74">
-        <v>175500000000</v>
+        <v>161500000000</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -5963,9 +5967,7 @@
       <c r="H141" s="57">
         <v>14000000000</v>
       </c>
-      <c r="I141" s="59">
-        <v>14000000000</v>
-      </c>
+      <c r="I141" s="58"/>
     </row>
     <row r="142" spans="1:9">
       <c r="A142" s="76"/>
@@ -6031,7 +6033,7 @@
         <v>7000000000</v>
       </c>
       <c r="I144" s="59">
-        <v>9000000000</v>
+        <v>11000000000</v>
       </c>
     </row>
     <row r="145" spans="1:9">
@@ -6073,7 +6075,7 @@
         <v>8000000000</v>
       </c>
       <c r="I146" s="59">
-        <v>11000000000</v>
+        <v>14000000000</v>
       </c>
     </row>
     <row r="147" spans="1:9">
@@ -6094,7 +6096,7 @@
         <v>8000000000</v>
       </c>
       <c r="I147" s="59">
-        <v>8000000000</v>
+        <v>10000000000</v>
       </c>
     </row>
     <row r="148" spans="1:9">
@@ -6157,7 +6159,7 @@
         <v>3000000000</v>
       </c>
       <c r="I150" s="59">
-        <v>5000000000</v>
+        <v>8000000000</v>
       </c>
     </row>
     <row r="151" spans="1:9">
@@ -6195,118 +6197,116 @@
       <c r="G152" s="52"/>
       <c r="H152" s="52"/>
       <c r="I152" s="59">
-        <v>3000000000</v>
+        <v>5000000000</v>
       </c>
     </row>
     <row r="153" spans="1:9">
-      <c r="A153" s="60"/>
-      <c r="B153" s="68" t="s">
+      <c r="A153" s="76"/>
+      <c r="B153" s="54" t="s">
+        <v>407</v>
+      </c>
+      <c r="C153" s="52"/>
+      <c r="D153" s="56" t="s">
+        <v>383</v>
+      </c>
+      <c r="E153" s="56" t="s">
+        <v>408</v>
+      </c>
+      <c r="F153" s="52"/>
+      <c r="G153" s="52"/>
+      <c r="H153" s="52"/>
+      <c r="I153" s="59">
+        <v>4000000000</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9">
+      <c r="A154" s="60"/>
+      <c r="B154" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C153" s="69" t="s">
+      <c r="C154" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D153" s="69" t="s">
+      <c r="D154" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E153" s="70" t="s">
+      <c r="E154" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F153" s="72">
+      <c r="F154" s="72">
         <v>108500000000</v>
       </c>
-      <c r="G153" s="72">
+      <c r="G154" s="72">
         <v>96000000000</v>
       </c>
-      <c r="H153" s="72">
+      <c r="H154" s="72">
         <v>106000000000</v>
       </c>
-      <c r="I153" s="74">
-        <v>110000000000</v>
-      </c>
-    </row>
-    <row r="154" spans="1:9">
-      <c r="A154" s="55" t="s">
-        <v>407</v>
-      </c>
-      <c r="B154" s="54" t="s">
-        <v>408</v>
-      </c>
-      <c r="C154" s="52"/>
-      <c r="D154" s="52"/>
-      <c r="E154" s="52"/>
-      <c r="F154" s="57">
-        <v>235000000</v>
-      </c>
-      <c r="G154" s="52"/>
-      <c r="H154" s="52"/>
-      <c r="I154" s="58"/>
+      <c r="I154" s="74">
+        <v>112000000000</v>
+      </c>
     </row>
     <row r="155" spans="1:9">
-      <c r="A155" s="76"/>
+      <c r="A155" s="55" t="s">
+        <v>409</v>
+      </c>
       <c r="B155" s="54" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C155" s="52"/>
       <c r="D155" s="52"/>
       <c r="E155" s="52"/>
       <c r="F155" s="57">
-        <v>162500000</v>
-      </c>
-      <c r="G155" s="57">
-        <v>162500000</v>
-      </c>
-      <c r="H155" s="57">
-        <v>50000000</v>
-      </c>
+        <v>235000000</v>
+      </c>
+      <c r="G155" s="52"/>
+      <c r="H155" s="52"/>
       <c r="I155" s="58"/>
     </row>
     <row r="156" spans="1:9">
       <c r="A156" s="76"/>
       <c r="B156" s="54" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C156" s="52"/>
       <c r="D156" s="52"/>
       <c r="E156" s="52"/>
       <c r="F156" s="57">
-        <v>100000000</v>
+        <v>162500000</v>
       </c>
       <c r="G156" s="57">
-        <v>100000000</v>
+        <v>162500000</v>
       </c>
       <c r="H156" s="57">
-        <v>100000000</v>
-      </c>
-      <c r="I156" s="59">
-        <v>100000000</v>
-      </c>
+        <v>50000000</v>
+      </c>
+      <c r="I156" s="58"/>
     </row>
     <row r="157" spans="1:9">
       <c r="A157" s="76"/>
       <c r="B157" s="54" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C157" s="52"/>
       <c r="D157" s="52"/>
       <c r="E157" s="52"/>
       <c r="F157" s="57">
-        <v>325000000</v>
+        <v>100000000</v>
       </c>
       <c r="G157" s="57">
-        <v>325000000</v>
+        <v>100000000</v>
       </c>
       <c r="H157" s="57">
-        <v>325000000</v>
+        <v>100000000</v>
       </c>
       <c r="I157" s="59">
-        <v>475000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="158" spans="1:9">
       <c r="A158" s="76"/>
       <c r="B158" s="54" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C158" s="52"/>
       <c r="D158" s="52"/>
@@ -6321,234 +6321,238 @@
         <v>325000000</v>
       </c>
       <c r="I158" s="59">
-        <v>360000000</v>
+        <v>475000000</v>
       </c>
     </row>
     <row r="159" spans="1:9">
       <c r="A159" s="76"/>
       <c r="B159" s="54" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C159" s="52"/>
       <c r="D159" s="52"/>
       <c r="E159" s="52"/>
       <c r="F159" s="57">
-        <v>355000000</v>
+        <v>325000000</v>
       </c>
       <c r="G159" s="57">
-        <v>355000000</v>
+        <v>325000000</v>
       </c>
       <c r="H159" s="57">
-        <v>355000000</v>
+        <v>325000000</v>
       </c>
       <c r="I159" s="59">
-        <v>355000000</v>
+        <v>475000000</v>
       </c>
     </row>
     <row r="160" spans="1:9">
       <c r="A160" s="76"/>
       <c r="B160" s="54" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C160" s="52"/>
       <c r="D160" s="52"/>
       <c r="E160" s="52"/>
       <c r="F160" s="57">
-        <v>380000000</v>
+        <v>355000000</v>
       </c>
       <c r="G160" s="57">
-        <v>380000000</v>
+        <v>355000000</v>
       </c>
       <c r="H160" s="57">
-        <v>380000000</v>
+        <v>355000000</v>
       </c>
       <c r="I160" s="59">
-        <v>381800000</v>
+        <v>555000000</v>
       </c>
     </row>
     <row r="161" spans="1:9">
       <c r="A161" s="76"/>
       <c r="B161" s="54" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C161" s="52"/>
       <c r="D161" s="52"/>
       <c r="E161" s="52"/>
       <c r="F161" s="57">
-        <v>350000000</v>
+        <v>380000000</v>
       </c>
       <c r="G161" s="57">
-        <v>350000000</v>
+        <v>380000000</v>
       </c>
       <c r="H161" s="57">
-        <v>350000000</v>
+        <v>380000000</v>
       </c>
       <c r="I161" s="59">
-        <v>350000000</v>
+        <v>381800000</v>
       </c>
     </row>
     <row r="162" spans="1:9">
       <c r="A162" s="76"/>
       <c r="B162" s="54" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C162" s="52"/>
       <c r="D162" s="52"/>
       <c r="E162" s="52"/>
       <c r="F162" s="57">
-        <v>793000000</v>
+        <v>350000000</v>
       </c>
       <c r="G162" s="57">
-        <v>793000000</v>
+        <v>350000000</v>
       </c>
       <c r="H162" s="57">
-        <v>793000000</v>
+        <v>350000000</v>
       </c>
       <c r="I162" s="59">
-        <v>793000000</v>
+        <v>350000000</v>
       </c>
     </row>
     <row r="163" spans="1:9">
       <c r="A163" s="76"/>
       <c r="B163" s="54" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C163" s="52"/>
       <c r="D163" s="52"/>
       <c r="E163" s="52"/>
       <c r="F163" s="57">
-        <v>731000000</v>
+        <v>793000000</v>
       </c>
       <c r="G163" s="57">
-        <v>731000000</v>
+        <v>793000000</v>
       </c>
       <c r="H163" s="57">
-        <v>731000000</v>
+        <v>793000000</v>
       </c>
       <c r="I163" s="59">
-        <v>731000000</v>
+        <v>793000000</v>
       </c>
     </row>
     <row r="164" spans="1:9">
       <c r="A164" s="76"/>
       <c r="B164" s="54" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C164" s="52"/>
       <c r="D164" s="52"/>
       <c r="E164" s="52"/>
       <c r="F164" s="57">
-        <v>85000000</v>
+        <v>731000000</v>
       </c>
       <c r="G164" s="57">
-        <v>85000000</v>
+        <v>731000000</v>
       </c>
       <c r="H164" s="57">
-        <v>85000000</v>
+        <v>731000000</v>
       </c>
       <c r="I164" s="59">
-        <v>85000000</v>
+        <v>731000000</v>
       </c>
     </row>
     <row r="165" spans="1:9">
       <c r="A165" s="76"/>
       <c r="B165" s="54" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C165" s="52"/>
       <c r="D165" s="52"/>
       <c r="E165" s="52"/>
       <c r="F165" s="57">
-        <v>224500000</v>
+        <v>85000000</v>
       </c>
       <c r="G165" s="57">
-        <v>224500000</v>
+        <v>85000000</v>
       </c>
       <c r="H165" s="57">
-        <v>224500000</v>
+        <v>85000000</v>
       </c>
       <c r="I165" s="59">
-        <v>224500000</v>
+        <v>85000000</v>
       </c>
     </row>
     <row r="166" spans="1:9">
       <c r="A166" s="76"/>
       <c r="B166" s="54" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C166" s="52"/>
       <c r="D166" s="52"/>
       <c r="E166" s="52"/>
       <c r="F166" s="57">
+        <v>224500000</v>
+      </c>
+      <c r="G166" s="57">
+        <v>224500000</v>
+      </c>
+      <c r="H166" s="57">
+        <v>224500000</v>
+      </c>
+      <c r="I166" s="59">
+        <v>224500000</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9">
+      <c r="A167" s="76"/>
+      <c r="B167" s="54" t="s">
+        <v>422</v>
+      </c>
+      <c r="C167" s="52"/>
+      <c r="D167" s="52"/>
+      <c r="E167" s="52"/>
+      <c r="F167" s="57">
         <v>64100000</v>
       </c>
-      <c r="G166" s="57">
+      <c r="G167" s="57">
         <v>64100000</v>
       </c>
-      <c r="H166" s="57">
+      <c r="H167" s="57">
         <v>64100000</v>
       </c>
-      <c r="I166" s="59">
+      <c r="I167" s="59">
         <v>64100000</v>
       </c>
     </row>
-    <row r="167" spans="1:9">
-      <c r="A167" s="60"/>
-      <c r="B167" s="68" t="s">
+    <row r="168" spans="1:9">
+      <c r="A168" s="60"/>
+      <c r="B168" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C167" s="69" t="s">
+      <c r="C168" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D167" s="69" t="s">
+      <c r="D168" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E167" s="70" t="s">
+      <c r="E168" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F167" s="72">
+      <c r="F168" s="72">
         <v>4130100000</v>
       </c>
-      <c r="G167" s="72">
+      <c r="G168" s="72">
         <v>3895100000</v>
       </c>
-      <c r="H167" s="72">
+      <c r="H168" s="72">
         <v>3782600000</v>
       </c>
-      <c r="I167" s="74">
-        <v>3919400000</v>
-      </c>
-    </row>
-    <row r="168" spans="1:9">
-      <c r="A168" s="55" t="s">
-        <v>421</v>
-      </c>
-      <c r="B168" s="54" t="s">
-        <v>422</v>
-      </c>
-      <c r="C168" s="52"/>
-      <c r="D168" s="56" t="s">
-        <v>74</v>
-      </c>
-      <c r="E168" s="56" t="s">
-        <v>75</v>
-      </c>
-      <c r="F168" s="52"/>
-      <c r="G168" s="52"/>
-      <c r="H168" s="52"/>
-      <c r="I168" s="58"/>
+      <c r="I168" s="74">
+        <v>4234400000</v>
+      </c>
     </row>
     <row r="169" spans="1:9">
-      <c r="A169" s="76"/>
+      <c r="A169" s="55" t="s">
+        <v>423</v>
+      </c>
       <c r="B169" s="54" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C169" s="52"/>
       <c r="D169" s="56" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E169" s="56" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F169" s="52"/>
       <c r="G169" s="52"/>
@@ -6558,14 +6562,14 @@
     <row r="170" spans="1:9">
       <c r="A170" s="76"/>
       <c r="B170" s="54" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C170" s="52"/>
       <c r="D170" s="56" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E170" s="56" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F170" s="52"/>
       <c r="G170" s="52"/>
@@ -6575,14 +6579,14 @@
     <row r="171" spans="1:9">
       <c r="A171" s="76"/>
       <c r="B171" s="54" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C171" s="52"/>
       <c r="D171" s="56" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E171" s="56" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F171" s="52"/>
       <c r="G171" s="52"/>
@@ -6592,14 +6596,14 @@
     <row r="172" spans="1:9">
       <c r="A172" s="76"/>
       <c r="B172" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C172" s="52"/>
       <c r="D172" s="56" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E172" s="56" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F172" s="52"/>
       <c r="G172" s="52"/>
@@ -6609,14 +6613,14 @@
     <row r="173" spans="1:9">
       <c r="A173" s="76"/>
       <c r="B173" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C173" s="52"/>
       <c r="D173" s="56" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E173" s="56" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F173" s="52"/>
       <c r="G173" s="52"/>
@@ -6626,14 +6630,14 @@
     <row r="174" spans="1:9">
       <c r="A174" s="76"/>
       <c r="B174" s="54" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C174" s="52"/>
       <c r="D174" s="56" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E174" s="56" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F174" s="52"/>
       <c r="G174" s="52"/>
@@ -6643,14 +6647,14 @@
     <row r="175" spans="1:9">
       <c r="A175" s="76"/>
       <c r="B175" s="54" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C175" s="52"/>
       <c r="D175" s="56" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E175" s="56" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F175" s="52"/>
       <c r="G175" s="52"/>
@@ -6660,14 +6664,14 @@
     <row r="176" spans="1:9">
       <c r="A176" s="76"/>
       <c r="B176" s="54" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C176" s="52"/>
       <c r="D176" s="56" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E176" s="56" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F176" s="52"/>
       <c r="G176" s="52"/>
@@ -6677,14 +6681,14 @@
     <row r="177" spans="1:9">
       <c r="A177" s="76"/>
       <c r="B177" s="54" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C177" s="52"/>
       <c r="D177" s="56" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E177" s="56" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F177" s="52"/>
       <c r="G177" s="52"/>
@@ -6694,14 +6698,14 @@
     <row r="178" spans="1:9">
       <c r="A178" s="76"/>
       <c r="B178" s="54" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C178" s="52"/>
       <c r="D178" s="56" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E178" s="56" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F178" s="52"/>
       <c r="G178" s="52"/>
@@ -6711,14 +6715,14 @@
     <row r="179" spans="1:9">
       <c r="A179" s="76"/>
       <c r="B179" s="54" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C179" s="52"/>
       <c r="D179" s="56" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E179" s="56" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F179" s="52"/>
       <c r="G179" s="52"/>
@@ -6728,14 +6732,14 @@
     <row r="180" spans="1:9">
       <c r="A180" s="76"/>
       <c r="B180" s="54" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C180" s="52"/>
       <c r="D180" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E180" s="56" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="F180" s="52"/>
       <c r="G180" s="52"/>
@@ -6745,14 +6749,14 @@
     <row r="181" spans="1:9">
       <c r="A181" s="76"/>
       <c r="B181" s="54" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C181" s="52"/>
       <c r="D181" s="56" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="E181" s="56" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="F181" s="52"/>
       <c r="G181" s="52"/>
@@ -6762,14 +6766,14 @@
     <row r="182" spans="1:9">
       <c r="A182" s="76"/>
       <c r="B182" s="54" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C182" s="52"/>
       <c r="D182" s="56" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E182" s="56" t="s">
-        <v>38</v>
+        <v>119</v>
       </c>
       <c r="F182" s="52"/>
       <c r="G182" s="52"/>
@@ -6779,14 +6783,14 @@
     <row r="183" spans="1:9">
       <c r="A183" s="76"/>
       <c r="B183" s="54" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C183" s="52"/>
       <c r="D183" s="56" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E183" s="56" t="s">
-        <v>129</v>
+        <v>38</v>
       </c>
       <c r="F183" s="52"/>
       <c r="G183" s="52"/>
@@ -6796,14 +6800,14 @@
     <row r="184" spans="1:9">
       <c r="A184" s="76"/>
       <c r="B184" s="54" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C184" s="52"/>
       <c r="D184" s="56" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E184" s="56" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F184" s="52"/>
       <c r="G184" s="52"/>
@@ -6811,54 +6815,54 @@
       <c r="I184" s="58"/>
     </row>
     <row r="185" spans="1:9">
-      <c r="A185" s="60"/>
-      <c r="B185" s="68" t="s">
+      <c r="A185" s="76"/>
+      <c r="B185" s="54" t="s">
+        <v>440</v>
+      </c>
+      <c r="C185" s="52"/>
+      <c r="D185" s="56" t="s">
+        <v>132</v>
+      </c>
+      <c r="E185" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="F185" s="52"/>
+      <c r="G185" s="52"/>
+      <c r="H185" s="52"/>
+      <c r="I185" s="58"/>
+    </row>
+    <row r="186" spans="1:9">
+      <c r="A186" s="60"/>
+      <c r="B186" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C185" s="69" t="s">
+      <c r="C186" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D185" s="69" t="s">
+      <c r="D186" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E185" s="70" t="s">
+      <c r="E186" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F185" s="71"/>
-      <c r="G185" s="71"/>
-      <c r="H185" s="71"/>
-      <c r="I185" s="73"/>
-    </row>
-    <row r="186" spans="1:9">
-      <c r="A186" s="55" t="s">
-        <v>439</v>
-      </c>
-      <c r="B186" s="54" t="s">
-        <v>440</v>
-      </c>
-      <c r="C186" s="52"/>
-      <c r="D186" s="56" t="s">
-        <v>148</v>
-      </c>
-      <c r="E186" s="56" t="s">
-        <v>149</v>
-      </c>
-      <c r="F186" s="52"/>
-      <c r="G186" s="52"/>
-      <c r="H186" s="52"/>
-      <c r="I186" s="58"/>
+      <c r="F186" s="71"/>
+      <c r="G186" s="71"/>
+      <c r="H186" s="71"/>
+      <c r="I186" s="73"/>
     </row>
     <row r="187" spans="1:9">
-      <c r="A187" s="76"/>
+      <c r="A187" s="55" t="s">
+        <v>441</v>
+      </c>
       <c r="B187" s="54" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C187" s="52"/>
       <c r="D187" s="56" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E187" s="56" t="s">
-        <v>43</v>
+        <v>149</v>
       </c>
       <c r="F187" s="52"/>
       <c r="G187" s="52"/>
@@ -6866,54 +6870,54 @@
       <c r="I187" s="58"/>
     </row>
     <row r="188" spans="1:9">
-      <c r="A188" s="60"/>
-      <c r="B188" s="68" t="s">
+      <c r="A188" s="76"/>
+      <c r="B188" s="54" t="s">
+        <v>443</v>
+      </c>
+      <c r="C188" s="52"/>
+      <c r="D188" s="56" t="s">
+        <v>151</v>
+      </c>
+      <c r="E188" s="56" t="s">
+        <v>43</v>
+      </c>
+      <c r="F188" s="52"/>
+      <c r="G188" s="52"/>
+      <c r="H188" s="52"/>
+      <c r="I188" s="58"/>
+    </row>
+    <row r="189" spans="1:9">
+      <c r="A189" s="60"/>
+      <c r="B189" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C188" s="69" t="s">
+      <c r="C189" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D188" s="69" t="s">
+      <c r="D189" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E188" s="70" t="s">
+      <c r="E189" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F188" s="71"/>
-      <c r="G188" s="71"/>
-      <c r="H188" s="71"/>
-      <c r="I188" s="73"/>
-    </row>
-    <row r="189" spans="1:9">
-      <c r="A189" s="55" t="s">
-        <v>442</v>
-      </c>
-      <c r="B189" s="54" t="s">
-        <v>443</v>
-      </c>
-      <c r="C189" s="52"/>
-      <c r="D189" s="56" t="s">
-        <v>154</v>
-      </c>
-      <c r="E189" s="56" t="s">
-        <v>155</v>
-      </c>
-      <c r="F189" s="52"/>
-      <c r="G189" s="52"/>
-      <c r="H189" s="52"/>
-      <c r="I189" s="58"/>
+      <c r="F189" s="71"/>
+      <c r="G189" s="71"/>
+      <c r="H189" s="71"/>
+      <c r="I189" s="73"/>
     </row>
     <row r="190" spans="1:9">
-      <c r="A190" s="76"/>
+      <c r="A190" s="55" t="s">
+        <v>444</v>
+      </c>
       <c r="B190" s="54" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C190" s="52"/>
       <c r="D190" s="56" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E190" s="56" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F190" s="52"/>
       <c r="G190" s="52"/>
@@ -6923,14 +6927,14 @@
     <row r="191" spans="1:9">
       <c r="A191" s="76"/>
       <c r="B191" s="54" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C191" s="52"/>
       <c r="D191" s="56" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E191" s="56" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F191" s="52"/>
       <c r="G191" s="52"/>
@@ -6940,14 +6944,14 @@
     <row r="192" spans="1:9">
       <c r="A192" s="76"/>
       <c r="B192" s="54" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C192" s="52"/>
       <c r="D192" s="56" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="E192" s="56" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="F192" s="52"/>
       <c r="G192" s="52"/>
@@ -6957,14 +6961,14 @@
     <row r="193" spans="1:9">
       <c r="A193" s="76"/>
       <c r="B193" s="54" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C193" s="52"/>
       <c r="D193" s="56" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E193" s="56" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F193" s="52"/>
       <c r="G193" s="52"/>
@@ -6974,14 +6978,14 @@
     <row r="194" spans="1:9">
       <c r="A194" s="76"/>
       <c r="B194" s="54" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C194" s="52"/>
       <c r="D194" s="56" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E194" s="56" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="F194" s="52"/>
       <c r="G194" s="52"/>
@@ -6991,14 +6995,14 @@
     <row r="195" spans="1:9">
       <c r="A195" s="76"/>
       <c r="B195" s="54" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C195" s="52"/>
       <c r="D195" s="56" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="E195" s="56" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F195" s="52"/>
       <c r="G195" s="52"/>
@@ -7008,14 +7012,14 @@
     <row r="196" spans="1:9">
       <c r="A196" s="76"/>
       <c r="B196" s="54" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C196" s="52"/>
       <c r="D196" s="56" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E196" s="56" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F196" s="52"/>
       <c r="G196" s="52"/>
@@ -7025,14 +7029,14 @@
     <row r="197" spans="1:9">
       <c r="A197" s="76"/>
       <c r="B197" s="54" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C197" s="52"/>
       <c r="D197" s="56" t="s">
-        <v>199</v>
+        <v>179</v>
       </c>
       <c r="E197" s="56" t="s">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="F197" s="52"/>
       <c r="G197" s="52"/>
@@ -7042,14 +7046,14 @@
     <row r="198" spans="1:9">
       <c r="A198" s="76"/>
       <c r="B198" s="54" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C198" s="52"/>
       <c r="D198" s="56" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E198" s="56" t="s">
-        <v>54</v>
+        <v>200</v>
       </c>
       <c r="F198" s="52"/>
       <c r="G198" s="52"/>
@@ -7059,14 +7063,14 @@
     <row r="199" spans="1:9">
       <c r="A199" s="76"/>
       <c r="B199" s="54" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C199" s="52"/>
       <c r="D199" s="56" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E199" s="56" t="s">
-        <v>205</v>
+        <v>54</v>
       </c>
       <c r="F199" s="52"/>
       <c r="G199" s="52"/>
@@ -7076,14 +7080,14 @@
     <row r="200" spans="1:9">
       <c r="A200" s="76"/>
       <c r="B200" s="54" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C200" s="52"/>
       <c r="D200" s="56" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="E200" s="56" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F200" s="52"/>
       <c r="G200" s="52"/>
@@ -7093,14 +7097,14 @@
     <row r="201" spans="1:9">
       <c r="A201" s="76"/>
       <c r="B201" s="54" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C201" s="52"/>
       <c r="D201" s="56" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E201" s="56" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F201" s="52"/>
       <c r="G201" s="52"/>
@@ -7110,14 +7114,14 @@
     <row r="202" spans="1:9">
       <c r="A202" s="76"/>
       <c r="B202" s="54" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C202" s="52"/>
       <c r="D202" s="56" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E202" s="56" t="s">
-        <v>58</v>
+        <v>212</v>
       </c>
       <c r="F202" s="52"/>
       <c r="G202" s="52"/>
@@ -7127,14 +7131,14 @@
     <row r="203" spans="1:9">
       <c r="A203" s="76"/>
       <c r="B203" s="54" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C203" s="52"/>
       <c r="D203" s="56" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E203" s="56" t="s">
-        <v>217</v>
+        <v>58</v>
       </c>
       <c r="F203" s="52"/>
       <c r="G203" s="52"/>
@@ -7144,14 +7148,14 @@
     <row r="204" spans="1:9">
       <c r="A204" s="76"/>
       <c r="B204" s="54" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C204" s="52"/>
       <c r="D204" s="56" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E204" s="56" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F204" s="52"/>
       <c r="G204" s="52"/>
@@ -7161,14 +7165,14 @@
     <row r="205" spans="1:9">
       <c r="A205" s="76"/>
       <c r="B205" s="54" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C205" s="52"/>
       <c r="D205" s="56" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="E205" s="56" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="F205" s="52"/>
       <c r="G205" s="52"/>
@@ -7176,54 +7180,54 @@
       <c r="I205" s="58"/>
     </row>
     <row r="206" spans="1:9">
-      <c r="A206" s="60"/>
-      <c r="B206" s="68" t="s">
+      <c r="A206" s="76"/>
+      <c r="B206" s="54" t="s">
+        <v>461</v>
+      </c>
+      <c r="C206" s="52"/>
+      <c r="D206" s="56" t="s">
+        <v>223</v>
+      </c>
+      <c r="E206" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="F206" s="52"/>
+      <c r="G206" s="52"/>
+      <c r="H206" s="52"/>
+      <c r="I206" s="58"/>
+    </row>
+    <row r="207" spans="1:9">
+      <c r="A207" s="60"/>
+      <c r="B207" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C206" s="69" t="s">
+      <c r="C207" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D206" s="69" t="s">
+      <c r="D207" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E206" s="70" t="s">
+      <c r="E207" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F206" s="71"/>
-      <c r="G206" s="71"/>
-      <c r="H206" s="71"/>
-      <c r="I206" s="73"/>
-    </row>
-    <row r="207" spans="1:9">
-      <c r="A207" s="55" t="s">
-        <v>460</v>
-      </c>
-      <c r="B207" s="54" t="s">
-        <v>461</v>
-      </c>
-      <c r="C207" s="52"/>
-      <c r="D207" s="56" t="s">
-        <v>233</v>
-      </c>
-      <c r="E207" s="56" t="s">
-        <v>234</v>
-      </c>
-      <c r="F207" s="52"/>
-      <c r="G207" s="52"/>
-      <c r="H207" s="52"/>
-      <c r="I207" s="58"/>
+      <c r="F207" s="71"/>
+      <c r="G207" s="71"/>
+      <c r="H207" s="71"/>
+      <c r="I207" s="73"/>
     </row>
     <row r="208" spans="1:9">
-      <c r="A208" s="76"/>
+      <c r="A208" s="55" t="s">
+        <v>462</v>
+      </c>
       <c r="B208" s="54" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C208" s="52"/>
       <c r="D208" s="56" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="E208" s="56" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="F208" s="52"/>
       <c r="G208" s="52"/>
@@ -7233,14 +7237,14 @@
     <row r="209" spans="1:9">
       <c r="A209" s="76"/>
       <c r="B209" s="54" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C209" s="52"/>
       <c r="D209" s="56" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E209" s="56" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="F209" s="52"/>
       <c r="G209" s="52"/>
@@ -7248,54 +7252,54 @@
       <c r="I209" s="58"/>
     </row>
     <row r="210" spans="1:9">
-      <c r="A210" s="60"/>
-      <c r="B210" s="68" t="s">
+      <c r="A210" s="76"/>
+      <c r="B210" s="54" t="s">
+        <v>465</v>
+      </c>
+      <c r="C210" s="52"/>
+      <c r="D210" s="56" t="s">
+        <v>240</v>
+      </c>
+      <c r="E210" s="56" t="s">
+        <v>241</v>
+      </c>
+      <c r="F210" s="52"/>
+      <c r="G210" s="52"/>
+      <c r="H210" s="52"/>
+      <c r="I210" s="58"/>
+    </row>
+    <row r="211" spans="1:9">
+      <c r="A211" s="60"/>
+      <c r="B211" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C210" s="69" t="s">
+      <c r="C211" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D210" s="69" t="s">
+      <c r="D211" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E210" s="70" t="s">
+      <c r="E211" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F210" s="71"/>
-      <c r="G210" s="71"/>
-      <c r="H210" s="71"/>
-      <c r="I210" s="73"/>
-    </row>
-    <row r="211" spans="1:9">
-      <c r="A211" s="55" t="s">
-        <v>464</v>
-      </c>
-      <c r="B211" s="54" t="s">
-        <v>465</v>
-      </c>
-      <c r="C211" s="52"/>
-      <c r="D211" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="E211" s="56" t="s">
+      <c r="F211" s="71"/>
+      <c r="G211" s="71"/>
+      <c r="H211" s="71"/>
+      <c r="I211" s="73"/>
+    </row>
+    <row r="212" spans="1:9">
+      <c r="A212" s="55" t="s">
         <v>466</v>
       </c>
-      <c r="F211" s="52"/>
-      <c r="G211" s="52"/>
-      <c r="H211" s="52"/>
-      <c r="I211" s="58"/>
-    </row>
-    <row r="212" spans="1:9">
-      <c r="A212" s="76"/>
       <c r="B212" s="54" t="s">
         <v>467</v>
       </c>
       <c r="C212" s="52"/>
       <c r="D212" s="56" t="s">
-        <v>154</v>
+        <v>78</v>
       </c>
       <c r="E212" s="56" t="s">
-        <v>155</v>
+        <v>468</v>
       </c>
       <c r="F212" s="52"/>
       <c r="G212" s="52"/>
@@ -7305,14 +7309,14 @@
     <row r="213" spans="1:9">
       <c r="A213" s="76"/>
       <c r="B213" s="54" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C213" s="52"/>
       <c r="D213" s="56" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E213" s="56" t="s">
-        <v>469</v>
+        <v>155</v>
       </c>
       <c r="F213" s="52"/>
       <c r="G213" s="52"/>
@@ -7326,10 +7330,10 @@
       </c>
       <c r="C214" s="52"/>
       <c r="D214" s="56" t="s">
-        <v>74</v>
+        <v>148</v>
       </c>
       <c r="E214" s="56" t="s">
-        <v>216</v>
+        <v>471</v>
       </c>
       <c r="F214" s="52"/>
       <c r="G214" s="52"/>
@@ -7339,14 +7343,14 @@
     <row r="215" spans="1:9">
       <c r="A215" s="76"/>
       <c r="B215" s="54" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C215" s="52"/>
       <c r="D215" s="56" t="s">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="E215" s="56" t="s">
-        <v>158</v>
+        <v>216</v>
       </c>
       <c r="F215" s="52"/>
       <c r="G215" s="52"/>
@@ -7356,14 +7360,14 @@
     <row r="216" spans="1:9">
       <c r="A216" s="76"/>
       <c r="B216" s="54" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C216" s="52"/>
       <c r="D216" s="56" t="s">
-        <v>233</v>
+        <v>114</v>
       </c>
       <c r="E216" s="56" t="s">
-        <v>473</v>
+        <v>158</v>
       </c>
       <c r="F216" s="52"/>
       <c r="G216" s="52"/>
@@ -7377,7 +7381,7 @@
       </c>
       <c r="C217" s="52"/>
       <c r="D217" s="56" t="s">
-        <v>78</v>
+        <v>233</v>
       </c>
       <c r="E217" s="56" t="s">
         <v>475</v>
@@ -7394,10 +7398,10 @@
       </c>
       <c r="C218" s="52"/>
       <c r="D218" s="56" t="s">
-        <v>160</v>
+        <v>78</v>
       </c>
       <c r="E218" s="56" t="s">
-        <v>161</v>
+        <v>477</v>
       </c>
       <c r="F218" s="52"/>
       <c r="G218" s="52"/>
@@ -7407,14 +7411,14 @@
     <row r="219" spans="1:9">
       <c r="A219" s="76"/>
       <c r="B219" s="54" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C219" s="52"/>
       <c r="D219" s="56" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="E219" s="56" t="s">
-        <v>478</v>
+        <v>161</v>
       </c>
       <c r="F219" s="52"/>
       <c r="G219" s="52"/>
@@ -7428,7 +7432,7 @@
       </c>
       <c r="C220" s="52"/>
       <c r="D220" s="56" t="s">
-        <v>74</v>
+        <v>148</v>
       </c>
       <c r="E220" s="56" t="s">
         <v>480</v>
@@ -7445,10 +7449,10 @@
       </c>
       <c r="C221" s="52"/>
       <c r="D221" s="56" t="s">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="E221" s="56" t="s">
-        <v>164</v>
+        <v>482</v>
       </c>
       <c r="F221" s="52"/>
       <c r="G221" s="52"/>
@@ -7458,14 +7462,14 @@
     <row r="222" spans="1:9">
       <c r="A222" s="76"/>
       <c r="B222" s="54" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C222" s="52"/>
       <c r="D222" s="56" t="s">
-        <v>233</v>
+        <v>114</v>
       </c>
       <c r="E222" s="56" t="s">
-        <v>483</v>
+        <v>164</v>
       </c>
       <c r="F222" s="52"/>
       <c r="G222" s="52"/>
@@ -7479,7 +7483,7 @@
       </c>
       <c r="C223" s="52"/>
       <c r="D223" s="56" t="s">
-        <v>78</v>
+        <v>233</v>
       </c>
       <c r="E223" s="56" t="s">
         <v>485</v>
@@ -7496,10 +7500,10 @@
       </c>
       <c r="C224" s="52"/>
       <c r="D224" s="56" t="s">
-        <v>167</v>
+        <v>78</v>
       </c>
       <c r="E224" s="56" t="s">
-        <v>168</v>
+        <v>487</v>
       </c>
       <c r="F224" s="52"/>
       <c r="G224" s="52"/>
@@ -7509,14 +7513,14 @@
     <row r="225" spans="1:9">
       <c r="A225" s="76"/>
       <c r="B225" s="54" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="C225" s="52"/>
       <c r="D225" s="56" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="E225" s="56" t="s">
-        <v>488</v>
+        <v>168</v>
       </c>
       <c r="F225" s="52"/>
       <c r="G225" s="52"/>
@@ -7530,10 +7534,10 @@
       </c>
       <c r="C226" s="52"/>
       <c r="D226" s="56" t="s">
-        <v>74</v>
+        <v>148</v>
       </c>
       <c r="E226" s="56" t="s">
-        <v>75</v>
+        <v>490</v>
       </c>
       <c r="F226" s="52"/>
       <c r="G226" s="52"/>
@@ -7543,14 +7547,14 @@
     <row r="227" spans="1:9">
       <c r="A227" s="76"/>
       <c r="B227" s="54" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C227" s="52"/>
       <c r="D227" s="56" t="s">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="E227" s="56" t="s">
-        <v>171</v>
+        <v>75</v>
       </c>
       <c r="F227" s="52"/>
       <c r="G227" s="52"/>
@@ -7560,14 +7564,14 @@
     <row r="228" spans="1:9">
       <c r="A228" s="76"/>
       <c r="B228" s="54" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C228" s="52"/>
       <c r="D228" s="56" t="s">
-        <v>233</v>
+        <v>114</v>
       </c>
       <c r="E228" s="56" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
       <c r="F228" s="52"/>
       <c r="G228" s="52"/>
@@ -7577,14 +7581,14 @@
     <row r="229" spans="1:9">
       <c r="A229" s="76"/>
       <c r="B229" s="54" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="C229" s="52"/>
       <c r="D229" s="56" t="s">
-        <v>78</v>
+        <v>233</v>
       </c>
       <c r="E229" s="56" t="s">
-        <v>79</v>
+        <v>228</v>
       </c>
       <c r="F229" s="52"/>
       <c r="G229" s="52"/>
@@ -7594,14 +7598,14 @@
     <row r="230" spans="1:9">
       <c r="A230" s="76"/>
       <c r="B230" s="54" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C230" s="52"/>
       <c r="D230" s="56" t="s">
-        <v>173</v>
+        <v>78</v>
       </c>
       <c r="E230" s="56" t="s">
-        <v>174</v>
+        <v>79</v>
       </c>
       <c r="F230" s="52"/>
       <c r="G230" s="52"/>
@@ -7611,14 +7615,14 @@
     <row r="231" spans="1:9">
       <c r="A231" s="76"/>
       <c r="B231" s="54" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C231" s="52"/>
       <c r="D231" s="56" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="E231" s="56" t="s">
-        <v>495</v>
+        <v>174</v>
       </c>
       <c r="F231" s="52"/>
       <c r="G231" s="52"/>
@@ -7632,10 +7636,10 @@
       </c>
       <c r="C232" s="52"/>
       <c r="D232" s="56" t="s">
-        <v>82</v>
+        <v>148</v>
       </c>
       <c r="E232" s="56" t="s">
-        <v>83</v>
+        <v>497</v>
       </c>
       <c r="F232" s="52"/>
       <c r="G232" s="52"/>
@@ -7645,14 +7649,14 @@
     <row r="233" spans="1:9">
       <c r="A233" s="76"/>
       <c r="B233" s="54" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C233" s="52"/>
       <c r="D233" s="56" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="E233" s="56" t="s">
-        <v>177</v>
+        <v>83</v>
       </c>
       <c r="F233" s="52"/>
       <c r="G233" s="52"/>
@@ -7662,14 +7666,14 @@
     <row r="234" spans="1:9">
       <c r="A234" s="76"/>
       <c r="B234" s="54" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="C234" s="52"/>
       <c r="D234" s="56" t="s">
-        <v>233</v>
+        <v>114</v>
       </c>
       <c r="E234" s="56" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="F234" s="52"/>
       <c r="G234" s="52"/>
@@ -7679,14 +7683,14 @@
     <row r="235" spans="1:9">
       <c r="A235" s="76"/>
       <c r="B235" s="54" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C235" s="52"/>
       <c r="D235" s="56" t="s">
-        <v>86</v>
+        <v>233</v>
       </c>
       <c r="E235" s="56" t="s">
-        <v>500</v>
+        <v>231</v>
       </c>
       <c r="F235" s="52"/>
       <c r="G235" s="52"/>
@@ -7700,10 +7704,10 @@
       </c>
       <c r="C236" s="52"/>
       <c r="D236" s="56" t="s">
-        <v>179</v>
+        <v>86</v>
       </c>
       <c r="E236" s="56" t="s">
-        <v>180</v>
+        <v>502</v>
       </c>
       <c r="F236" s="52"/>
       <c r="G236" s="52"/>
@@ -7713,14 +7717,14 @@
     <row r="237" spans="1:9">
       <c r="A237" s="76"/>
       <c r="B237" s="54" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C237" s="52"/>
       <c r="D237" s="56" t="s">
-        <v>148</v>
+        <v>179</v>
       </c>
       <c r="E237" s="56" t="s">
-        <v>503</v>
+        <v>180</v>
       </c>
       <c r="F237" s="52"/>
       <c r="G237" s="52"/>
@@ -7734,7 +7738,7 @@
       </c>
       <c r="C238" s="52"/>
       <c r="D238" s="56" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="E238" s="56" t="s">
         <v>505</v>
@@ -7751,10 +7755,10 @@
       </c>
       <c r="C239" s="52"/>
       <c r="D239" s="56" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="E239" s="56" t="s">
-        <v>183</v>
+        <v>507</v>
       </c>
       <c r="F239" s="52"/>
       <c r="G239" s="52"/>
@@ -7764,14 +7768,14 @@
     <row r="240" spans="1:9">
       <c r="A240" s="76"/>
       <c r="B240" s="54" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C240" s="52"/>
       <c r="D240" s="56" t="s">
-        <v>233</v>
+        <v>114</v>
       </c>
       <c r="E240" s="56" t="s">
-        <v>234</v>
+        <v>183</v>
       </c>
       <c r="F240" s="52"/>
       <c r="G240" s="52"/>
@@ -7781,14 +7785,14 @@
     <row r="241" spans="1:9">
       <c r="A241" s="76"/>
       <c r="B241" s="54" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="C241" s="52"/>
       <c r="D241" s="56" t="s">
-        <v>86</v>
+        <v>233</v>
       </c>
       <c r="E241" s="56" t="s">
-        <v>87</v>
+        <v>234</v>
       </c>
       <c r="F241" s="52"/>
       <c r="G241" s="52"/>
@@ -7798,14 +7802,14 @@
     <row r="242" spans="1:9">
       <c r="A242" s="76"/>
       <c r="B242" s="54" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C242" s="52"/>
       <c r="D242" s="56" t="s">
-        <v>202</v>
+        <v>86</v>
       </c>
       <c r="E242" s="56" t="s">
-        <v>186</v>
+        <v>87</v>
       </c>
       <c r="F242" s="52"/>
       <c r="G242" s="52"/>
@@ -7815,14 +7819,14 @@
     <row r="243" spans="1:9">
       <c r="A243" s="76"/>
       <c r="B243" s="54" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C243" s="52"/>
       <c r="D243" s="56" t="s">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="E243" s="56" t="s">
-        <v>511</v>
+        <v>186</v>
       </c>
       <c r="F243" s="52"/>
       <c r="G243" s="52"/>
@@ -7836,7 +7840,7 @@
       </c>
       <c r="C244" s="52"/>
       <c r="D244" s="56" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="E244" s="56" t="s">
         <v>513</v>
@@ -7853,10 +7857,10 @@
       </c>
       <c r="C245" s="52"/>
       <c r="D245" s="56" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="E245" s="56" t="s">
-        <v>47</v>
+        <v>515</v>
       </c>
       <c r="F245" s="52"/>
       <c r="G245" s="52"/>
@@ -7866,14 +7870,14 @@
     <row r="246" spans="1:9">
       <c r="A246" s="76"/>
       <c r="B246" s="54" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C246" s="52"/>
       <c r="D246" s="56" t="s">
-        <v>237</v>
+        <v>114</v>
       </c>
       <c r="E246" s="56" t="s">
-        <v>238</v>
+        <v>47</v>
       </c>
       <c r="F246" s="52"/>
       <c r="G246" s="52"/>
@@ -7883,14 +7887,14 @@
     <row r="247" spans="1:9">
       <c r="A247" s="76"/>
       <c r="B247" s="54" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C247" s="52"/>
       <c r="D247" s="56" t="s">
-        <v>90</v>
+        <v>237</v>
       </c>
       <c r="E247" s="56" t="s">
-        <v>91</v>
+        <v>238</v>
       </c>
       <c r="F247" s="52"/>
       <c r="G247" s="52"/>
@@ -7900,14 +7904,14 @@
     <row r="248" spans="1:9">
       <c r="A248" s="76"/>
       <c r="B248" s="54" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C248" s="52"/>
       <c r="D248" s="56" t="s">
-        <v>202</v>
+        <v>90</v>
       </c>
       <c r="E248" s="56" t="s">
-        <v>191</v>
+        <v>91</v>
       </c>
       <c r="F248" s="52"/>
       <c r="G248" s="52"/>
@@ -7917,14 +7921,14 @@
     <row r="249" spans="1:9">
       <c r="A249" s="76"/>
       <c r="B249" s="54" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C249" s="52"/>
       <c r="D249" s="56" t="s">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="E249" s="56" t="s">
-        <v>519</v>
+        <v>191</v>
       </c>
       <c r="F249" s="52"/>
       <c r="G249" s="52"/>
@@ -7938,7 +7942,7 @@
       </c>
       <c r="C250" s="52"/>
       <c r="D250" s="56" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="E250" s="56" t="s">
         <v>521</v>
@@ -7955,10 +7959,10 @@
       </c>
       <c r="C251" s="52"/>
       <c r="D251" s="56" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="E251" s="56" t="s">
-        <v>50</v>
+        <v>523</v>
       </c>
       <c r="F251" s="52"/>
       <c r="G251" s="52"/>
@@ -7968,14 +7972,14 @@
     <row r="252" spans="1:9">
       <c r="A252" s="76"/>
       <c r="B252" s="54" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C252" s="52"/>
       <c r="D252" s="56" t="s">
-        <v>240</v>
+        <v>114</v>
       </c>
       <c r="E252" s="56" t="s">
-        <v>524</v>
+        <v>50</v>
       </c>
       <c r="F252" s="52"/>
       <c r="G252" s="52"/>
@@ -7989,7 +7993,7 @@
       </c>
       <c r="C253" s="52"/>
       <c r="D253" s="56" t="s">
-        <v>97</v>
+        <v>240</v>
       </c>
       <c r="E253" s="56" t="s">
         <v>526</v>
@@ -8006,10 +8010,10 @@
       </c>
       <c r="C254" s="52"/>
       <c r="D254" s="56" t="s">
-        <v>202</v>
+        <v>97</v>
       </c>
       <c r="E254" s="56" t="s">
-        <v>196</v>
+        <v>528</v>
       </c>
       <c r="F254" s="52"/>
       <c r="G254" s="52"/>
@@ -8019,14 +8023,14 @@
     <row r="255" spans="1:9">
       <c r="A255" s="76"/>
       <c r="B255" s="54" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C255" s="52"/>
       <c r="D255" s="56" t="s">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="E255" s="56" t="s">
-        <v>529</v>
+        <v>196</v>
       </c>
       <c r="F255" s="52"/>
       <c r="G255" s="52"/>
@@ -8040,7 +8044,7 @@
       </c>
       <c r="C256" s="52"/>
       <c r="D256" s="56" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="E256" s="56" t="s">
         <v>531</v>
@@ -8057,10 +8061,10 @@
       </c>
       <c r="C257" s="52"/>
       <c r="D257" s="56" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="E257" s="56" t="s">
-        <v>200</v>
+        <v>533</v>
       </c>
       <c r="F257" s="52"/>
       <c r="G257" s="52"/>
@@ -8070,14 +8074,14 @@
     <row r="258" spans="1:9">
       <c r="A258" s="76"/>
       <c r="B258" s="54" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="C258" s="52"/>
       <c r="D258" s="56" t="s">
-        <v>240</v>
+        <v>114</v>
       </c>
       <c r="E258" s="56" t="s">
-        <v>241</v>
+        <v>200</v>
       </c>
       <c r="F258" s="52"/>
       <c r="G258" s="52"/>
@@ -8087,14 +8091,14 @@
     <row r="259" spans="1:9">
       <c r="A259" s="76"/>
       <c r="B259" s="54" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C259" s="52"/>
       <c r="D259" s="56" t="s">
-        <v>97</v>
+        <v>240</v>
       </c>
       <c r="E259" s="56" t="s">
-        <v>535</v>
+        <v>241</v>
       </c>
       <c r="F259" s="52"/>
       <c r="G259" s="52"/>
@@ -8108,10 +8112,10 @@
       </c>
       <c r="C260" s="52"/>
       <c r="D260" s="56" t="s">
-        <v>202</v>
+        <v>97</v>
       </c>
       <c r="E260" s="56" t="s">
-        <v>54</v>
+        <v>537</v>
       </c>
       <c r="F260" s="52"/>
       <c r="G260" s="52"/>
@@ -8121,14 +8125,14 @@
     <row r="261" spans="1:9">
       <c r="A261" s="76"/>
       <c r="B261" s="54" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C261" s="52"/>
       <c r="D261" s="56" t="s">
-        <v>148</v>
+        <v>202</v>
       </c>
       <c r="E261" s="56" t="s">
-        <v>538</v>
+        <v>54</v>
       </c>
       <c r="F261" s="52"/>
       <c r="G261" s="52"/>
@@ -8142,7 +8146,7 @@
       </c>
       <c r="C262" s="52"/>
       <c r="D262" s="56" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="E262" s="56" t="s">
         <v>540</v>
@@ -8159,10 +8163,10 @@
       </c>
       <c r="C263" s="52"/>
       <c r="D263" s="56" t="s">
+        <v>93</v>
+      </c>
+      <c r="E263" s="56" t="s">
         <v>542</v>
-      </c>
-      <c r="E263" s="56" t="s">
-        <v>205</v>
       </c>
       <c r="F263" s="52"/>
       <c r="G263" s="52"/>
@@ -8176,7 +8180,7 @@
       </c>
       <c r="C264" s="52"/>
       <c r="D264" s="56" t="s">
-        <v>114</v>
+        <v>544</v>
       </c>
       <c r="E264" s="56" t="s">
         <v>205</v>
@@ -8189,14 +8193,14 @@
     <row r="265" spans="1:9">
       <c r="A265" s="76"/>
       <c r="B265" s="54" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C265" s="52"/>
       <c r="D265" s="56" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="E265" s="56" t="s">
-        <v>545</v>
+        <v>205</v>
       </c>
       <c r="F265" s="52"/>
       <c r="G265" s="52"/>
@@ -8210,10 +8214,10 @@
       </c>
       <c r="C266" s="52"/>
       <c r="D266" s="56" t="s">
-        <v>208</v>
+        <v>97</v>
       </c>
       <c r="E266" s="56" t="s">
-        <v>209</v>
+        <v>547</v>
       </c>
       <c r="F266" s="52"/>
       <c r="G266" s="52"/>
@@ -8223,14 +8227,14 @@
     <row r="267" spans="1:9">
       <c r="A267" s="76"/>
       <c r="B267" s="54" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C267" s="52"/>
       <c r="D267" s="56" t="s">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="E267" s="56" t="s">
-        <v>548</v>
+        <v>209</v>
       </c>
       <c r="F267" s="52"/>
       <c r="G267" s="52"/>
@@ -8244,10 +8248,10 @@
       </c>
       <c r="C268" s="52"/>
       <c r="D268" s="56" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="E268" s="56" t="s">
-        <v>94</v>
+        <v>550</v>
       </c>
       <c r="F268" s="52"/>
       <c r="G268" s="52"/>
@@ -8257,14 +8261,14 @@
     <row r="269" spans="1:9">
       <c r="A269" s="76"/>
       <c r="B269" s="54" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C269" s="52"/>
       <c r="D269" s="56" t="s">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="E269" s="56" t="s">
-        <v>212</v>
+        <v>94</v>
       </c>
       <c r="F269" s="52"/>
       <c r="G269" s="52"/>
@@ -8274,14 +8278,14 @@
     <row r="270" spans="1:9">
       <c r="A270" s="76"/>
       <c r="B270" s="54" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C270" s="52"/>
       <c r="D270" s="56" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="E270" s="56" t="s">
-        <v>552</v>
+        <v>212</v>
       </c>
       <c r="F270" s="52"/>
       <c r="G270" s="52"/>
@@ -8295,10 +8299,10 @@
       </c>
       <c r="C271" s="52"/>
       <c r="D271" s="56" t="s">
-        <v>214</v>
+        <v>97</v>
       </c>
       <c r="E271" s="56" t="s">
-        <v>58</v>
+        <v>554</v>
       </c>
       <c r="F271" s="52"/>
       <c r="G271" s="52"/>
@@ -8308,14 +8312,14 @@
     <row r="272" spans="1:9">
       <c r="A272" s="76"/>
       <c r="B272" s="54" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="C272" s="52"/>
       <c r="D272" s="56" t="s">
-        <v>148</v>
+        <v>214</v>
       </c>
       <c r="E272" s="56" t="s">
-        <v>142</v>
+        <v>58</v>
       </c>
       <c r="F272" s="52"/>
       <c r="G272" s="52"/>
@@ -8325,14 +8329,14 @@
     <row r="273" spans="1:9">
       <c r="A273" s="76"/>
       <c r="B273" s="54" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C273" s="52"/>
       <c r="D273" s="56" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
       <c r="E273" s="56" t="s">
-        <v>556</v>
+        <v>142</v>
       </c>
       <c r="F273" s="52"/>
       <c r="G273" s="52"/>
@@ -8346,10 +8350,10 @@
       </c>
       <c r="C274" s="52"/>
       <c r="D274" s="56" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E274" s="56" t="s">
-        <v>217</v>
+        <v>558</v>
       </c>
       <c r="F274" s="52"/>
       <c r="G274" s="52"/>
@@ -8359,14 +8363,14 @@
     <row r="275" spans="1:9">
       <c r="A275" s="76"/>
       <c r="B275" s="54" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="C275" s="52"/>
       <c r="D275" s="56" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="E275" s="56" t="s">
-        <v>559</v>
+        <v>217</v>
       </c>
       <c r="F275" s="52"/>
       <c r="G275" s="52"/>
@@ -8380,10 +8384,10 @@
       </c>
       <c r="C276" s="52"/>
       <c r="D276" s="56" t="s">
-        <v>219</v>
+        <v>97</v>
       </c>
       <c r="E276" s="56" t="s">
-        <v>220</v>
+        <v>561</v>
       </c>
       <c r="F276" s="52"/>
       <c r="G276" s="52"/>
@@ -8393,14 +8397,14 @@
     <row r="277" spans="1:9">
       <c r="A277" s="76"/>
       <c r="B277" s="54" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C277" s="52"/>
       <c r="D277" s="56" t="s">
-        <v>148</v>
+        <v>219</v>
       </c>
       <c r="E277" s="56" t="s">
-        <v>145</v>
+        <v>220</v>
       </c>
       <c r="F277" s="52"/>
       <c r="G277" s="52"/>
@@ -8410,14 +8414,14 @@
     <row r="278" spans="1:9">
       <c r="A278" s="76"/>
       <c r="B278" s="54" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C278" s="52"/>
       <c r="D278" s="56" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
       <c r="E278" s="56" t="s">
-        <v>563</v>
+        <v>145</v>
       </c>
       <c r="F278" s="52"/>
       <c r="G278" s="52"/>
@@ -8431,10 +8435,10 @@
       </c>
       <c r="C279" s="52"/>
       <c r="D279" s="56" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E279" s="56" t="s">
-        <v>224</v>
+        <v>565</v>
       </c>
       <c r="F279" s="52"/>
       <c r="G279" s="52"/>
@@ -8444,14 +8448,14 @@
     <row r="280" spans="1:9">
       <c r="A280" s="76"/>
       <c r="B280" s="54" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C280" s="52"/>
       <c r="D280" s="56" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="E280" s="56" t="s">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="F280" s="52"/>
       <c r="G280" s="52"/>
@@ -8461,14 +8465,14 @@
     <row r="281" spans="1:9">
       <c r="A281" s="76"/>
       <c r="B281" s="54" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C281" s="52"/>
       <c r="D281" s="56" t="s">
-        <v>148</v>
+        <v>97</v>
       </c>
       <c r="E281" s="56" t="s">
-        <v>567</v>
+        <v>98</v>
       </c>
       <c r="F281" s="52"/>
       <c r="G281" s="52"/>
@@ -8482,7 +8486,7 @@
       </c>
       <c r="C282" s="52"/>
       <c r="D282" s="56" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
       <c r="E282" s="56" t="s">
         <v>569</v>
@@ -8499,7 +8503,7 @@
       </c>
       <c r="C283" s="52"/>
       <c r="D283" s="56" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E283" s="56" t="s">
         <v>571</v>
@@ -8516,10 +8520,10 @@
       </c>
       <c r="C284" s="52"/>
       <c r="D284" s="56" t="s">
-        <v>148</v>
+        <v>114</v>
       </c>
       <c r="E284" s="56" t="s">
-        <v>149</v>
+        <v>573</v>
       </c>
       <c r="F284" s="52"/>
       <c r="G284" s="52"/>
@@ -8529,14 +8533,14 @@
     <row r="285" spans="1:9">
       <c r="A285" s="76"/>
       <c r="B285" s="54" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C285" s="52"/>
       <c r="D285" s="56" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
       <c r="E285" s="56" t="s">
-        <v>574</v>
+        <v>149</v>
       </c>
       <c r="F285" s="52"/>
       <c r="G285" s="52"/>
@@ -8550,7 +8554,7 @@
       </c>
       <c r="C286" s="52"/>
       <c r="D286" s="56" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E286" s="56" t="s">
         <v>576</v>
@@ -8567,7 +8571,7 @@
       </c>
       <c r="C287" s="52"/>
       <c r="D287" s="56" t="s">
-        <v>151</v>
+        <v>114</v>
       </c>
       <c r="E287" s="56" t="s">
         <v>578</v>
@@ -8584,10 +8588,10 @@
       </c>
       <c r="C288" s="52"/>
       <c r="D288" s="56" t="s">
-        <v>101</v>
+        <v>151</v>
       </c>
       <c r="E288" s="56" t="s">
-        <v>102</v>
+        <v>580</v>
       </c>
       <c r="F288" s="52"/>
       <c r="G288" s="52"/>
@@ -8597,14 +8601,14 @@
     <row r="289" spans="1:9">
       <c r="A289" s="76"/>
       <c r="B289" s="54" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C289" s="52"/>
       <c r="D289" s="56" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E289" s="56" t="s">
-        <v>581</v>
+        <v>102</v>
       </c>
       <c r="F289" s="52"/>
       <c r="G289" s="52"/>
@@ -8618,7 +8622,7 @@
       </c>
       <c r="C290" s="52"/>
       <c r="D290" s="56" t="s">
-        <v>151</v>
+        <v>114</v>
       </c>
       <c r="E290" s="56" t="s">
         <v>583</v>
@@ -8635,10 +8639,10 @@
       </c>
       <c r="C291" s="52"/>
       <c r="D291" s="56" t="s">
-        <v>104</v>
+        <v>151</v>
       </c>
       <c r="E291" s="56" t="s">
-        <v>105</v>
+        <v>585</v>
       </c>
       <c r="F291" s="52"/>
       <c r="G291" s="52"/>
@@ -8648,14 +8652,14 @@
     <row r="292" spans="1:9">
       <c r="A292" s="76"/>
       <c r="B292" s="54" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C292" s="52"/>
       <c r="D292" s="56" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E292" s="56" t="s">
-        <v>586</v>
+        <v>105</v>
       </c>
       <c r="F292" s="52"/>
       <c r="G292" s="52"/>
@@ -8669,10 +8673,10 @@
       </c>
       <c r="C293" s="52"/>
       <c r="D293" s="56" t="s">
-        <v>151</v>
+        <v>114</v>
       </c>
       <c r="E293" s="56" t="s">
-        <v>43</v>
+        <v>588</v>
       </c>
       <c r="F293" s="52"/>
       <c r="G293" s="52"/>
@@ -8682,14 +8686,14 @@
     <row r="294" spans="1:9">
       <c r="A294" s="76"/>
       <c r="B294" s="54" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C294" s="52"/>
       <c r="D294" s="56" t="s">
-        <v>108</v>
+        <v>151</v>
       </c>
       <c r="E294" s="56" t="s">
-        <v>589</v>
+        <v>43</v>
       </c>
       <c r="F294" s="52"/>
       <c r="G294" s="52"/>
@@ -8703,7 +8707,7 @@
       </c>
       <c r="C295" s="52"/>
       <c r="D295" s="56" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E295" s="56" t="s">
         <v>591</v>
@@ -8720,7 +8724,7 @@
       </c>
       <c r="C296" s="52"/>
       <c r="D296" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E296" s="56" t="s">
         <v>593</v>
@@ -8737,10 +8741,10 @@
       </c>
       <c r="C297" s="52"/>
       <c r="D297" s="56" t="s">
-        <v>108</v>
+        <v>137</v>
       </c>
       <c r="E297" s="56" t="s">
-        <v>109</v>
+        <v>595</v>
       </c>
       <c r="F297" s="52"/>
       <c r="G297" s="52"/>
@@ -8750,14 +8754,14 @@
     <row r="298" spans="1:9">
       <c r="A298" s="76"/>
       <c r="B298" s="54" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C298" s="52"/>
       <c r="D298" s="56" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E298" s="56" t="s">
-        <v>596</v>
+        <v>109</v>
       </c>
       <c r="F298" s="52"/>
       <c r="G298" s="52"/>
@@ -8771,7 +8775,7 @@
       </c>
       <c r="C299" s="52"/>
       <c r="D299" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E299" s="56" t="s">
         <v>598</v>
@@ -8788,7 +8792,7 @@
       </c>
       <c r="C300" s="52"/>
       <c r="D300" s="56" t="s">
-        <v>111</v>
+        <v>137</v>
       </c>
       <c r="E300" s="56" t="s">
         <v>600</v>
@@ -8805,7 +8809,7 @@
       </c>
       <c r="C301" s="52"/>
       <c r="D301" s="56" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E301" s="56" t="s">
         <v>602</v>
@@ -8822,7 +8826,7 @@
       </c>
       <c r="C302" s="52"/>
       <c r="D302" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E302" s="56" t="s">
         <v>604</v>
@@ -8839,10 +8843,10 @@
       </c>
       <c r="C303" s="52"/>
       <c r="D303" s="56" t="s">
-        <v>111</v>
+        <v>137</v>
       </c>
       <c r="E303" s="56" t="s">
-        <v>112</v>
+        <v>606</v>
       </c>
       <c r="F303" s="52"/>
       <c r="G303" s="52"/>
@@ -8852,14 +8856,14 @@
     <row r="304" spans="1:9">
       <c r="A304" s="76"/>
       <c r="B304" s="54" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C304" s="52"/>
       <c r="D304" s="56" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E304" s="56" t="s">
-        <v>607</v>
+        <v>112</v>
       </c>
       <c r="F304" s="52"/>
       <c r="G304" s="52"/>
@@ -8873,7 +8877,7 @@
       </c>
       <c r="C305" s="52"/>
       <c r="D305" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E305" s="56" t="s">
         <v>609</v>
@@ -8890,7 +8894,7 @@
       </c>
       <c r="C306" s="52"/>
       <c r="D306" s="56" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="E306" s="56" t="s">
         <v>611</v>
@@ -8907,7 +8911,7 @@
       </c>
       <c r="C307" s="52"/>
       <c r="D307" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E307" s="56" t="s">
         <v>613</v>
@@ -8924,10 +8928,10 @@
       </c>
       <c r="C308" s="52"/>
       <c r="D308" s="56" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="E308" s="56" t="s">
-        <v>115</v>
+        <v>615</v>
       </c>
       <c r="F308" s="52"/>
       <c r="G308" s="52"/>
@@ -8937,14 +8941,14 @@
     <row r="309" spans="1:9">
       <c r="A309" s="76"/>
       <c r="B309" s="54" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C309" s="52"/>
       <c r="D309" s="56" t="s">
-        <v>137</v>
+        <v>114</v>
       </c>
       <c r="E309" s="56" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="F309" s="52"/>
       <c r="G309" s="52"/>
@@ -8954,14 +8958,14 @@
     <row r="310" spans="1:9">
       <c r="A310" s="76"/>
       <c r="B310" s="54" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C310" s="52"/>
       <c r="D310" s="56" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="E310" s="56" t="s">
-        <v>617</v>
+        <v>138</v>
       </c>
       <c r="F310" s="52"/>
       <c r="G310" s="52"/>
@@ -8978,7 +8982,7 @@
         <v>118</v>
       </c>
       <c r="E311" s="56" t="s">
-        <v>119</v>
+        <v>619</v>
       </c>
       <c r="F311" s="52"/>
       <c r="G311" s="52"/>
@@ -8988,14 +8992,14 @@
     <row r="312" spans="1:9">
       <c r="A312" s="76"/>
       <c r="B312" s="54" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C312" s="52"/>
       <c r="D312" s="56" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E312" s="56" t="s">
-        <v>620</v>
+        <v>119</v>
       </c>
       <c r="F312" s="52"/>
       <c r="G312" s="52"/>
@@ -9012,7 +9016,7 @@
         <v>126</v>
       </c>
       <c r="E313" s="56" t="s">
-        <v>34</v>
+        <v>622</v>
       </c>
       <c r="F313" s="52"/>
       <c r="G313" s="52"/>
@@ -9022,14 +9026,14 @@
     <row r="314" spans="1:9">
       <c r="A314" s="76"/>
       <c r="B314" s="54" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="C314" s="52"/>
       <c r="D314" s="56" t="s">
         <v>126</v>
       </c>
       <c r="E314" s="56" t="s">
-        <v>623</v>
+        <v>34</v>
       </c>
       <c r="F314" s="52"/>
       <c r="G314" s="52"/>
@@ -9046,7 +9050,7 @@
         <v>126</v>
       </c>
       <c r="E315" s="56" t="s">
-        <v>124</v>
+        <v>625</v>
       </c>
       <c r="F315" s="52"/>
       <c r="G315" s="52"/>
@@ -9056,14 +9060,14 @@
     <row r="316" spans="1:9">
       <c r="A316" s="76"/>
       <c r="B316" s="54" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C316" s="52"/>
       <c r="D316" s="56" t="s">
         <v>126</v>
       </c>
       <c r="E316" s="56" t="s">
-        <v>38</v>
+        <v>124</v>
       </c>
       <c r="F316" s="52"/>
       <c r="G316" s="52"/>
@@ -9073,14 +9077,14 @@
     <row r="317" spans="1:9">
       <c r="A317" s="76"/>
       <c r="B317" s="54" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C317" s="52"/>
       <c r="D317" s="56" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E317" s="56" t="s">
-        <v>129</v>
+        <v>38</v>
       </c>
       <c r="F317" s="52"/>
       <c r="G317" s="52"/>
@@ -9090,14 +9094,14 @@
     <row r="318" spans="1:9">
       <c r="A318" s="76"/>
       <c r="B318" s="54" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C318" s="52"/>
       <c r="D318" s="56" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E318" s="56" t="s">
-        <v>628</v>
+        <v>129</v>
       </c>
       <c r="F318" s="52"/>
       <c r="G318" s="52"/>
@@ -9114,7 +9118,7 @@
         <v>132</v>
       </c>
       <c r="E319" s="56" t="s">
-        <v>133</v>
+        <v>630</v>
       </c>
       <c r="F319" s="52"/>
       <c r="G319" s="52"/>
@@ -9122,43 +9126,60 @@
       <c r="I319" s="58"/>
     </row>
     <row r="320" spans="1:9">
-      <c r="A320" s="60"/>
-      <c r="B320" s="68" t="s">
+      <c r="A320" s="76"/>
+      <c r="B320" s="54" t="s">
+        <v>631</v>
+      </c>
+      <c r="C320" s="52"/>
+      <c r="D320" s="56" t="s">
+        <v>132</v>
+      </c>
+      <c r="E320" s="56" t="s">
+        <v>133</v>
+      </c>
+      <c r="F320" s="52"/>
+      <c r="G320" s="52"/>
+      <c r="H320" s="52"/>
+      <c r="I320" s="58"/>
+    </row>
+    <row r="321" spans="1:9">
+      <c r="A321" s="60"/>
+      <c r="B321" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C320" s="69" t="s">
+      <c r="C321" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="D320" s="69" t="s">
+      <c r="D321" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="E320" s="70" t="s">
+      <c r="E321" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="F320" s="71"/>
-      <c r="G320" s="71"/>
-      <c r="H320" s="71"/>
-      <c r="I320" s="73"/>
-    </row>
-    <row r="321" spans="1:9">
-      <c r="A321" s="80" t="s">
-        <v>630</v>
-      </c>
-      <c r="B321" s="30"/>
-      <c r="C321" s="30"/>
-      <c r="D321" s="30"/>
-      <c r="E321" s="30"/>
-      <c r="F321" s="84">
+      <c r="F321" s="71"/>
+      <c r="G321" s="71"/>
+      <c r="H321" s="71"/>
+      <c r="I321" s="73"/>
+    </row>
+    <row r="322" spans="1:9">
+      <c r="A322" s="80" t="s">
+        <v>632</v>
+      </c>
+      <c r="B322" s="30"/>
+      <c r="C322" s="30"/>
+      <c r="D322" s="30"/>
+      <c r="E322" s="30"/>
+      <c r="F322" s="84">
         <v>1886130100000</v>
       </c>
-      <c r="G321" s="84">
+      <c r="G322" s="84">
         <v>1973895100000</v>
       </c>
-      <c r="H321" s="84">
+      <c r="H322" s="84">
         <v>2055582600000</v>
       </c>
-      <c r="I321" s="86">
-        <v>2094219400000</v>
+      <c r="I322" s="86">
+        <v>2104534400000</v>
       </c>
     </row>
   </sheetData>
@@ -9184,15 +9205,15 @@
     <mergeCell ref="A85:A90"/>
     <mergeCell ref="A91:A105"/>
     <mergeCell ref="A106:A121"/>
-    <mergeCell ref="A122:A153"/>
-    <mergeCell ref="A154:A167"/>
-    <mergeCell ref="A168:A185"/>
-    <mergeCell ref="A186:A188"/>
-    <mergeCell ref="A189:A206"/>
-    <mergeCell ref="A207:A210"/>
-    <mergeCell ref="A211:A320"/>
-    <mergeCell ref="A321:E321"/>
-    <mergeCell ref="A322:I322"/>
+    <mergeCell ref="A122:A154"/>
+    <mergeCell ref="A155:A168"/>
+    <mergeCell ref="A169:A186"/>
+    <mergeCell ref="A187:A189"/>
+    <mergeCell ref="A190:A207"/>
+    <mergeCell ref="A208:A211"/>
+    <mergeCell ref="A212:A321"/>
+    <mergeCell ref="A322:E322"/>
+    <mergeCell ref="A323:I323"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>